<commit_message>
Fix: bounds logic, improved greedy, L02 search, optimality certificates, Excel validation
- Fix Problem 1 bound/gap: upper_bound=1.0, gap=0.99% (was incorrectly 0%)
- Fix Problem 2 bound: properly labeled as loose relaxation bound
- Add improved_greedy pattern generator with candidate position tracking
- Add exact_enumeration, exact_geometry_cp, certificate modules
- Add L02 specialized search (l02_best_patterns.csv, l02_search_report.json)
- Add exact certificate infrastructure (NOT_PROVED due to computational limits)
- Fix Excel writer: separate template mappings, backup, validation report
- Fix 3D layout path to outputs/figures/3d_layouts/
- Add timing breakdowns to JSON/CSV/Excel
- Add ablation_results.csv, sensitivity_results.csv, seed_stability_results.csv
- Rewrite CLAUDE.md with comprehensive documentation
- Generate optimality_certificate_report.md with honest proof status

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/results/result1_filled.xlsx
+++ b/outputs/results/result1_filled.xlsx
@@ -1459,24 +1459,24 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G36"/>
+  <dimension ref="A1:G45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="18" customWidth="1" style="7" min="1" max="1"/>
-    <col width="18" customWidth="1" style="7" min="2" max="2"/>
-    <col width="18" customWidth="1" style="7" min="3" max="3"/>
-    <col width="18" customWidth="1" style="7" min="4" max="4"/>
-    <col width="18" customWidth="1" style="7" min="5" max="5"/>
-    <col width="18" customWidth="1" style="7" min="6" max="6"/>
-    <col width="18" customWidth="1" style="7" min="7" max="7"/>
-    <col width="18" customWidth="1" style="7" min="8" max="8"/>
-    <col width="18" customWidth="1" style="7" min="9" max="9"/>
+    <col width="22" customWidth="1" style="7" min="1" max="1"/>
+    <col width="22" customWidth="1" style="7" min="2" max="2"/>
+    <col width="22" customWidth="1" style="7" min="3" max="3"/>
+    <col width="22" customWidth="1" style="7" min="4" max="4"/>
+    <col width="22" customWidth="1" style="7" min="5" max="5"/>
+    <col width="22" customWidth="1" style="7" min="6" max="6"/>
+    <col width="22" customWidth="1" style="7" min="7" max="7"/>
+    <col width="22" customWidth="1" style="7" min="8" max="8"/>
+    <col width="22" customWidth="1" style="7" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="11" t="inlineStr">
         <is>
-          <t>Solution Summary - PROBLEM1</t>
+          <t>Computed Solution - PROBLEM1</t>
         </is>
       </c>
     </row>
@@ -1529,8 +1529,10 @@
           <t>Total Used Volume</t>
         </is>
       </c>
-      <c r="B7" s="14" t="n">
-        <v>75000000</v>
+      <c r="B7" s="14" t="inlineStr">
+        <is>
+          <t>75,000,000</t>
+        </is>
       </c>
     </row>
     <row r="8">
@@ -1539,8 +1541,10 @@
           <t>Total Waste Volume</t>
         </is>
       </c>
-      <c r="B8" s="14" t="n">
-        <v>750000</v>
+      <c r="B8" s="14" t="inlineStr">
+        <is>
+          <t>750,000</t>
+        </is>
       </c>
     </row>
     <row r="9">
@@ -1549,8 +1553,10 @@
           <t>Total Material Volume</t>
         </is>
       </c>
-      <c r="B9" s="14" t="n">
-        <v>75750000</v>
+      <c r="B9" s="14" t="inlineStr">
+        <is>
+          <t>75,750,000</t>
+        </is>
       </c>
     </row>
     <row r="10">
@@ -1568,475 +1574,566 @@
     <row r="11">
       <c r="A11" s="13" t="inlineStr">
         <is>
-          <t>Solve Time (s)</t>
+          <t>Waste Gap Ratio</t>
         </is>
       </c>
       <c r="B11" s="14" t="inlineStr">
         <is>
-          <t>0.03</t>
+          <t>0.9901%</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="13" t="inlineStr">
         <is>
-          <t>Upper Bound</t>
+          <t>Utilization Gap to 100%</t>
         </is>
       </c>
       <c r="B12" s="14" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>0.9901%</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="13" t="inlineStr">
         <is>
-          <t>Lower Bound</t>
+          <t>Upper Bound (utilization)</t>
         </is>
       </c>
       <c r="B13" s="14" t="inlineStr">
         <is>
-          <t>750000.00</t>
+          <t>1.0 (100%)</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="13" t="inlineStr">
         <is>
+          <t>Lower Bound</t>
+        </is>
+      </c>
+      <c r="B14" s="14" t="inlineStr">
+        <is>
+          <t>0.9901</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="13" t="inlineStr">
+        <is>
           <t>Gap</t>
         </is>
       </c>
-      <c r="B14" s="14" t="inlineStr">
-        <is>
-          <t>0.00%</t>
+      <c r="B15" s="14" t="inlineStr">
+        <is>
+          <t>0.9901%</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="12" t="inlineStr">
+      <c r="A16" s="13" t="inlineStr">
+        <is>
+          <t>Solve Time (s)</t>
+        </is>
+      </c>
+      <c r="B16" s="14" t="inlineStr">
+        <is>
+          <t>0.18</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="13" t="inlineStr">
+        <is>
+          <t>Optimality Note</t>
+        </is>
+      </c>
+      <c r="B17" s="14" t="inlineStr">
+        <is>
+          <t>Pattern-library optimal (not necessarily global optimal without complete pattern enumeration)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="12" t="inlineStr">
+        <is>
+          <t>Runtime Breakdown</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="13" t="inlineStr">
+        <is>
+          <t>pattern_generation_time</t>
+        </is>
+      </c>
+      <c r="B20" s="14" t="inlineStr">
+        <is>
+          <t>1.87s</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="13" t="inlineStr">
+        <is>
+          <t>master_solve_time</t>
+        </is>
+      </c>
+      <c r="B21" s="14" t="inlineStr">
+        <is>
+          <t>1.99s</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="13" t="inlineStr">
+        <is>
+          <t>plotting_time_problem1</t>
+        </is>
+      </c>
+      <c r="B22" s="14" t="inlineStr">
+        <is>
+          <t>13.38s</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="13" t="inlineStr">
+        <is>
+          <t>plotting_time_problem2</t>
+        </is>
+      </c>
+      <c r="B23" s="14" t="inlineStr">
+        <is>
+          <t>22.28s</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="12" t="inlineStr">
         <is>
           <t>Piece Production Quantities</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="15" t="inlineStr">
+    <row r="26">
+      <c r="A26" s="15" t="inlineStr">
         <is>
           <t>Piece</t>
         </is>
       </c>
-      <c r="B17" s="15" t="inlineStr">
+      <c r="B26" s="15" t="inlineStr">
         <is>
           <t>Quantity</t>
         </is>
       </c>
-      <c r="C17" s="15" t="inlineStr">
+      <c r="C26" s="15" t="inlineStr">
         <is>
           <t>Volume/Unit</t>
         </is>
       </c>
-      <c r="D17" s="15" t="inlineStr">
+      <c r="D26" s="15" t="inlineStr">
         <is>
           <t>Total Volume</t>
         </is>
       </c>
-      <c r="E17" s="15" t="inlineStr">
+      <c r="E26" s="15" t="inlineStr">
         <is>
           <t>Unit Profit</t>
         </is>
       </c>
-      <c r="F17" s="15" t="inlineStr">
+      <c r="F26" s="15" t="inlineStr">
         <is>
           <t>Total Profit</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="14" t="inlineStr">
+    <row r="27">
+      <c r="A27" s="14" t="inlineStr">
         <is>
           <t>J01</t>
         </is>
       </c>
-      <c r="B18" s="14" t="n">
+      <c r="B27" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="C18" s="14" t="n">
+      <c r="C27" s="14" t="n">
         <v>64000</v>
       </c>
-      <c r="D18" s="14" t="n">
+      <c r="D27" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="E18" s="14" t="n">
+      <c r="E27" s="14" t="n">
         <v>620</v>
       </c>
-      <c r="F18" s="14" t="n">
+      <c r="F27" s="14" t="n">
         <v>0</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="14" t="inlineStr">
-        <is>
-          <t>J02</t>
-        </is>
-      </c>
-      <c r="B19" s="14" t="n">
-        <v>150</v>
-      </c>
-      <c r="C19" s="14" t="n">
-        <v>80000</v>
-      </c>
-      <c r="D19" s="14" t="n">
-        <v>12000000</v>
-      </c>
-      <c r="E19" s="14" t="n">
-        <v>780</v>
-      </c>
-      <c r="F19" s="14" t="n">
-        <v>117000</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="14" t="inlineStr">
-        <is>
-          <t>J03</t>
-        </is>
-      </c>
-      <c r="B20" s="14" t="n">
-        <v>700</v>
-      </c>
-      <c r="C20" s="14" t="n">
-        <v>90000</v>
-      </c>
-      <c r="D20" s="14" t="n">
-        <v>63000000</v>
-      </c>
-      <c r="E20" s="14" t="n">
-        <v>880</v>
-      </c>
-      <c r="F20" s="14" t="n">
-        <v>616000</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="14" t="inlineStr">
-        <is>
-          <t>J04</t>
-        </is>
-      </c>
-      <c r="B21" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="C21" s="14" t="n">
-        <v>180000</v>
-      </c>
-      <c r="D21" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="E21" s="14" t="n">
-        <v>1850</v>
-      </c>
-      <c r="F21" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="14" t="inlineStr">
-        <is>
-          <t>J05</t>
-        </is>
-      </c>
-      <c r="B22" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="C22" s="14" t="n">
-        <v>240000</v>
-      </c>
-      <c r="D22" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="E22" s="14" t="n">
-        <v>2520</v>
-      </c>
-      <c r="F22" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="14" t="inlineStr">
-        <is>
-          <t>J06</t>
-        </is>
-      </c>
-      <c r="B23" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="C23" s="14" t="n">
-        <v>100000</v>
-      </c>
-      <c r="D23" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="E23" s="14" t="n">
-        <v>1000</v>
-      </c>
-      <c r="F23" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="14" t="inlineStr">
-        <is>
-          <t>J07</t>
-        </is>
-      </c>
-      <c r="B24" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="C24" s="14" t="n">
-        <v>48000</v>
-      </c>
-      <c r="D24" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="E24" s="14" t="n">
-        <v>540</v>
-      </c>
-      <c r="F24" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="12" t="inlineStr">
-        <is>
-          <t>Material Utilization Breakdown</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="15" t="inlineStr">
-        <is>
-          <t>Material</t>
-        </is>
-      </c>
-      <c r="B27" s="15" t="inlineStr">
-        <is>
-          <t>Count</t>
-        </is>
-      </c>
-      <c r="C27" s="15" t="inlineStr">
-        <is>
-          <t>Volume/Material</t>
-        </is>
-      </c>
-      <c r="D27" s="15" t="inlineStr">
-        <is>
-          <t>Total Volume</t>
-        </is>
-      </c>
-      <c r="E27" s="15" t="inlineStr">
-        <is>
-          <t>Used Volume</t>
-        </is>
-      </c>
-      <c r="F27" s="15" t="inlineStr">
-        <is>
-          <t>Waste</t>
-        </is>
-      </c>
-      <c r="G27" s="15" t="inlineStr">
-        <is>
-          <t>Utilization</t>
-        </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="14" t="inlineStr">
         <is>
-          <t>L01</t>
+          <t>J02</t>
         </is>
       </c>
       <c r="B28" s="14" t="n">
-        <v>5</v>
+        <v>150</v>
       </c>
       <c r="C28" s="14" t="n">
-        <v>9000000</v>
+        <v>80000</v>
       </c>
       <c r="D28" s="14" t="n">
-        <v>45000000</v>
+        <v>12000000</v>
       </c>
       <c r="E28" s="14" t="n">
-        <v>45000000</v>
+        <v>780</v>
       </c>
       <c r="F28" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="G28" s="14" t="inlineStr">
-        <is>
-          <t>100.00%</t>
-        </is>
+        <v>117000</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="14" t="inlineStr">
         <is>
-          <t>L02</t>
+          <t>J03</t>
         </is>
       </c>
       <c r="B29" s="14" t="n">
-        <v>5</v>
+        <v>700</v>
       </c>
       <c r="C29" s="14" t="n">
-        <v>3750000</v>
+        <v>90000</v>
       </c>
       <c r="D29" s="14" t="n">
-        <v>18750000</v>
+        <v>63000000</v>
       </c>
       <c r="E29" s="14" t="n">
-        <v>18000000</v>
+        <v>880</v>
       </c>
       <c r="F29" s="14" t="n">
-        <v>750000</v>
-      </c>
-      <c r="G29" s="14" t="inlineStr">
-        <is>
-          <t>96.00%</t>
-        </is>
+        <v>616000</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="14" t="inlineStr">
         <is>
-          <t>L03</t>
+          <t>J04</t>
         </is>
       </c>
       <c r="B30" s="14" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="C30" s="14" t="n">
-        <v>2400000</v>
+        <v>180000</v>
       </c>
       <c r="D30" s="14" t="n">
-        <v>12000000</v>
+        <v>0</v>
       </c>
       <c r="E30" s="14" t="n">
-        <v>12000000</v>
+        <v>1850</v>
       </c>
       <c r="F30" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="G30" s="14" t="inlineStr">
+    </row>
+    <row r="31">
+      <c r="A31" s="14" t="inlineStr">
+        <is>
+          <t>J05</t>
+        </is>
+      </c>
+      <c r="B31" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="C31" s="14" t="n">
+        <v>240000</v>
+      </c>
+      <c r="D31" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E31" s="14" t="n">
+        <v>2520</v>
+      </c>
+      <c r="F31" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="14" t="inlineStr">
+        <is>
+          <t>J06</t>
+        </is>
+      </c>
+      <c r="B32" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="C32" s="14" t="n">
+        <v>100000</v>
+      </c>
+      <c r="D32" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E32" s="14" t="n">
+        <v>1000</v>
+      </c>
+      <c r="F32" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="14" t="inlineStr">
+        <is>
+          <t>J07</t>
+        </is>
+      </c>
+      <c r="B33" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="C33" s="14" t="n">
+        <v>48000</v>
+      </c>
+      <c r="D33" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E33" s="14" t="n">
+        <v>540</v>
+      </c>
+      <c r="F33" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="12" t="inlineStr">
+        <is>
+          <t>Material Utilization Breakdown</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="15" t="inlineStr">
+        <is>
+          <t>Material</t>
+        </is>
+      </c>
+      <c r="B36" s="15" t="inlineStr">
+        <is>
+          <t>Count</t>
+        </is>
+      </c>
+      <c r="C36" s="15" t="inlineStr">
+        <is>
+          <t>Volume/Material</t>
+        </is>
+      </c>
+      <c r="D36" s="15" t="inlineStr">
+        <is>
+          <t>Total Volume</t>
+        </is>
+      </c>
+      <c r="E36" s="15" t="inlineStr">
+        <is>
+          <t>Used Volume</t>
+        </is>
+      </c>
+      <c r="F36" s="15" t="inlineStr">
+        <is>
+          <t>Waste</t>
+        </is>
+      </c>
+      <c r="G36" s="15" t="inlineStr">
+        <is>
+          <t>Utilization</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="14" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="B37" s="14" t="n">
+        <v>5</v>
+      </c>
+      <c r="C37" s="14" t="n">
+        <v>9000000</v>
+      </c>
+      <c r="D37" s="14" t="n">
+        <v>45000000</v>
+      </c>
+      <c r="E37" s="14" t="n">
+        <v>45000000</v>
+      </c>
+      <c r="F37" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G37" s="14" t="inlineStr">
         <is>
           <t>100.00%</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="12" t="inlineStr">
+    <row r="38">
+      <c r="A38" s="14" t="inlineStr">
+        <is>
+          <t>L02</t>
+        </is>
+      </c>
+      <c r="B38" s="14" t="n">
+        <v>5</v>
+      </c>
+      <c r="C38" s="14" t="n">
+        <v>3750000</v>
+      </c>
+      <c r="D38" s="14" t="n">
+        <v>18750000</v>
+      </c>
+      <c r="E38" s="14" t="n">
+        <v>18000000</v>
+      </c>
+      <c r="F38" s="14" t="n">
+        <v>750000</v>
+      </c>
+      <c r="G38" s="14" t="inlineStr">
+        <is>
+          <t>96.00%</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="14" t="inlineStr">
+        <is>
+          <t>L03</t>
+        </is>
+      </c>
+      <c r="B39" s="14" t="n">
+        <v>5</v>
+      </c>
+      <c r="C39" s="14" t="n">
+        <v>2400000</v>
+      </c>
+      <c r="D39" s="14" t="n">
+        <v>12000000</v>
+      </c>
+      <c r="E39" s="14" t="n">
+        <v>12000000</v>
+      </c>
+      <c r="F39" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G39" s="14" t="inlineStr">
+        <is>
+          <t>100.00%</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="12" t="inlineStr">
         <is>
           <t>Pattern Usage Details</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="15" t="inlineStr">
+    <row r="42">
+      <c r="A42" s="15" t="inlineStr">
         <is>
           <t>Pattern ID</t>
         </is>
       </c>
-      <c r="B33" s="15" t="inlineStr">
+      <c r="B42" s="15" t="inlineStr">
         <is>
           <t>Material</t>
         </is>
       </c>
-      <c r="C33" s="15" t="inlineStr">
+      <c r="C42" s="15" t="inlineStr">
         <is>
           <t>Times Used</t>
         </is>
       </c>
-      <c r="D33" s="15" t="inlineStr">
+      <c r="D42" s="15" t="inlineStr">
         <is>
           <t>Pieces</t>
         </is>
       </c>
-      <c r="E33" s="15" t="inlineStr">
+      <c r="E42" s="15" t="inlineStr">
         <is>
           <t>Used Volume</t>
         </is>
       </c>
-      <c r="F33" s="15" t="inlineStr">
+      <c r="F42" s="15" t="inlineStr">
         <is>
           <t>Utilization</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="14" t="n">
+    <row r="43">
+      <c r="A43" s="14" t="n">
         <v>13</v>
       </c>
-      <c r="B34" s="14" t="inlineStr">
+      <c r="B43" s="14" t="inlineStr">
         <is>
           <t>L01</t>
         </is>
       </c>
-      <c r="C34" s="14" t="n">
+      <c r="C43" s="14" t="n">
         <v>5</v>
       </c>
-      <c r="D34" s="14" t="n">
+      <c r="D43" s="14" t="n">
         <v>100</v>
       </c>
-      <c r="E34" s="14" t="n">
+      <c r="E43" s="14" t="n">
         <v>9000000</v>
       </c>
-      <c r="F34" s="14" t="inlineStr">
+      <c r="F43" s="14" t="inlineStr">
         <is>
           <t>100.00%</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="14" t="n">
-        <v>97</v>
-      </c>
-      <c r="B35" s="14" t="inlineStr">
+    <row r="44">
+      <c r="A44" s="14" t="n">
+        <v>90</v>
+      </c>
+      <c r="B44" s="14" t="inlineStr">
         <is>
           <t>L02</t>
         </is>
       </c>
-      <c r="C35" s="14" t="n">
+      <c r="C44" s="14" t="n">
         <v>5</v>
       </c>
-      <c r="D35" s="14" t="n">
+      <c r="D44" s="14" t="n">
         <v>40</v>
       </c>
-      <c r="E35" s="14" t="n">
+      <c r="E44" s="14" t="n">
         <v>3600000</v>
       </c>
-      <c r="F35" s="14" t="inlineStr">
+      <c r="F44" s="14" t="inlineStr">
         <is>
           <t>96.00%</t>
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="14" t="n">
-        <v>167</v>
-      </c>
-      <c r="B36" s="14" t="inlineStr">
+    <row r="45">
+      <c r="A45" s="14" t="n">
+        <v>153</v>
+      </c>
+      <c r="B45" s="14" t="inlineStr">
         <is>
           <t>L03</t>
         </is>
       </c>
-      <c r="C36" s="14" t="n">
+      <c r="C45" s="14" t="n">
         <v>5</v>
       </c>
-      <c r="D36" s="14" t="n">
+      <c r="D45" s="14" t="n">
         <v>30</v>
       </c>
-      <c r="E36" s="14" t="n">
+      <c r="E45" s="14" t="n">
         <v>2400000</v>
       </c>
-      <c r="F36" s="14" t="inlineStr">
+      <c r="F45" s="14" t="inlineStr">
         <is>
           <t>100.00%</t>
         </is>

</xml_diff>

<commit_message>
Fix: recover Problem 2 745680, Excel template filling for both files, combined validation
- Recover Problem 2 profit from 742400 to 745680 by reverting greedy.mode to legacy
- Fix Excel writer: detect theme-based grey fills, fill per-block piece counts
- Both result1_filled.xlsx and result2_filled.xlsx now 105/105 cells filled
- Combined excel_validation_report.json with result1 and result2 sections
- Fix ablation_results.csv with proper values
- Restore original result1.xlsx and result2.xlsx templates from git

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/results/result1_filled.xlsx
+++ b/outputs/results/result1_filled.xlsx
@@ -1144,7 +1144,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I18"/>
+  <dimension ref="B2:K19"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14"/>
   <cols>
     <col width="10.9636363636364" customWidth="1" style="7" min="2" max="2"/>
@@ -1208,13 +1208,27 @@
           <t>L01</t>
         </is>
       </c>
-      <c r="C4" s="6" t="n"/>
-      <c r="D4" s="6" t="n"/>
-      <c r="E4" s="6" t="n"/>
-      <c r="F4" s="6" t="n"/>
-      <c r="G4" s="6" t="n"/>
-      <c r="H4" s="6" t="n"/>
-      <c r="I4" s="6" t="n"/>
+      <c r="C4" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D4" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" s="6" t="n">
+        <v>100</v>
+      </c>
+      <c r="F4" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" s="6" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="5" ht="17" customHeight="1" s="7">
       <c r="B5" s="5" t="inlineStr">
@@ -1222,13 +1236,27 @@
           <t>L01</t>
         </is>
       </c>
-      <c r="C5" s="6" t="n"/>
-      <c r="D5" s="6" t="n"/>
-      <c r="E5" s="6" t="n"/>
-      <c r="F5" s="6" t="n"/>
-      <c r="G5" s="6" t="n"/>
-      <c r="H5" s="6" t="n"/>
-      <c r="I5" s="6" t="n"/>
+      <c r="C5" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D5" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" s="6" t="n">
+        <v>100</v>
+      </c>
+      <c r="F5" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" s="6" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="6" ht="17" customHeight="1" s="7">
       <c r="B6" s="5" t="inlineStr">
@@ -1236,13 +1264,27 @@
           <t>L01</t>
         </is>
       </c>
-      <c r="C6" s="6" t="n"/>
-      <c r="D6" s="6" t="n"/>
-      <c r="E6" s="6" t="n"/>
-      <c r="F6" s="6" t="n"/>
-      <c r="G6" s="6" t="n"/>
-      <c r="H6" s="6" t="n"/>
-      <c r="I6" s="6" t="n"/>
+      <c r="C6" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" s="6" t="n">
+        <v>100</v>
+      </c>
+      <c r="F6" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" s="6" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="7" ht="17" customHeight="1" s="7">
       <c r="B7" s="5" t="inlineStr">
@@ -1250,13 +1292,27 @@
           <t>L01</t>
         </is>
       </c>
-      <c r="C7" s="6" t="n"/>
-      <c r="D7" s="6" t="n"/>
-      <c r="E7" s="6" t="n"/>
-      <c r="F7" s="6" t="n"/>
-      <c r="G7" s="6" t="n"/>
-      <c r="H7" s="6" t="n"/>
-      <c r="I7" s="6" t="n"/>
+      <c r="C7" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" s="6" t="n">
+        <v>100</v>
+      </c>
+      <c r="F7" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" s="6" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="8" ht="17" customHeight="1" s="7">
       <c r="B8" s="5" t="inlineStr">
@@ -1264,13 +1320,27 @@
           <t>L01</t>
         </is>
       </c>
-      <c r="C8" s="6" t="n"/>
-      <c r="D8" s="6" t="n"/>
-      <c r="E8" s="6" t="n"/>
-      <c r="F8" s="6" t="n"/>
-      <c r="G8" s="6" t="n"/>
-      <c r="H8" s="6" t="n"/>
-      <c r="I8" s="6" t="n"/>
+      <c r="C8" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D8" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" s="6" t="n">
+        <v>100</v>
+      </c>
+      <c r="F8" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" s="6" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="9" ht="17" customHeight="1" s="7">
       <c r="B9" s="5" t="inlineStr">
@@ -1278,13 +1348,27 @@
           <t>L02</t>
         </is>
       </c>
-      <c r="C9" s="6" t="n"/>
-      <c r="D9" s="6" t="n"/>
-      <c r="E9" s="6" t="n"/>
-      <c r="F9" s="6" t="n"/>
-      <c r="G9" s="6" t="n"/>
-      <c r="H9" s="6" t="n"/>
-      <c r="I9" s="6" t="n"/>
+      <c r="C9" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D9" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" s="6" t="n">
+        <v>40</v>
+      </c>
+      <c r="F9" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" s="6" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="10" ht="17" customHeight="1" s="7">
       <c r="B10" s="5" t="inlineStr">
@@ -1292,13 +1376,27 @@
           <t>L02</t>
         </is>
       </c>
-      <c r="C10" s="6" t="n"/>
-      <c r="D10" s="6" t="n"/>
-      <c r="E10" s="6" t="n"/>
-      <c r="F10" s="6" t="n"/>
-      <c r="G10" s="6" t="n"/>
-      <c r="H10" s="6" t="n"/>
-      <c r="I10" s="6" t="n"/>
+      <c r="C10" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D10" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" s="6" t="n">
+        <v>40</v>
+      </c>
+      <c r="F10" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I10" s="6" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="11" ht="17" customHeight="1" s="7">
       <c r="B11" s="5" t="inlineStr">
@@ -1306,13 +1404,27 @@
           <t>L02</t>
         </is>
       </c>
-      <c r="C11" s="6" t="n"/>
-      <c r="D11" s="6" t="n"/>
-      <c r="E11" s="6" t="n"/>
-      <c r="F11" s="6" t="n"/>
-      <c r="G11" s="6" t="n"/>
-      <c r="H11" s="6" t="n"/>
-      <c r="I11" s="6" t="n"/>
+      <c r="C11" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D11" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" s="6" t="n">
+        <v>40</v>
+      </c>
+      <c r="F11" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I11" s="6" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="12" ht="17" customHeight="1" s="7">
       <c r="B12" s="5" t="inlineStr">
@@ -1320,13 +1432,27 @@
           <t>L02</t>
         </is>
       </c>
-      <c r="C12" s="6" t="n"/>
-      <c r="D12" s="6" t="n"/>
-      <c r="E12" s="6" t="n"/>
-      <c r="F12" s="6" t="n"/>
-      <c r="G12" s="6" t="n"/>
-      <c r="H12" s="6" t="n"/>
-      <c r="I12" s="6" t="n"/>
+      <c r="C12" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D12" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" s="6" t="n">
+        <v>40</v>
+      </c>
+      <c r="F12" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I12" s="6" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="13" ht="17" customHeight="1" s="7">
       <c r="B13" s="5" t="inlineStr">
@@ -1334,13 +1460,27 @@
           <t>L02</t>
         </is>
       </c>
-      <c r="C13" s="6" t="n"/>
-      <c r="D13" s="6" t="n"/>
-      <c r="E13" s="6" t="n"/>
-      <c r="F13" s="6" t="n"/>
-      <c r="G13" s="6" t="n"/>
-      <c r="H13" s="6" t="n"/>
-      <c r="I13" s="6" t="n"/>
+      <c r="C13" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D13" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E13" s="6" t="n">
+        <v>40</v>
+      </c>
+      <c r="F13" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G13" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I13" s="6" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="14" ht="17" customHeight="1" s="7">
       <c r="B14" s="5" t="inlineStr">
@@ -1348,13 +1488,27 @@
           <t>L03</t>
         </is>
       </c>
-      <c r="C14" s="6" t="n"/>
-      <c r="D14" s="6" t="n"/>
-      <c r="E14" s="6" t="n"/>
-      <c r="F14" s="6" t="n"/>
-      <c r="G14" s="6" t="n"/>
-      <c r="H14" s="6" t="n"/>
-      <c r="I14" s="6" t="n"/>
+      <c r="C14" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D14" s="6" t="n">
+        <v>30</v>
+      </c>
+      <c r="E14" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I14" s="6" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="15" ht="17" customHeight="1" s="7">
       <c r="B15" s="5" t="inlineStr">
@@ -1362,13 +1516,27 @@
           <t>L03</t>
         </is>
       </c>
-      <c r="C15" s="6" t="n"/>
-      <c r="D15" s="6" t="n"/>
-      <c r="E15" s="6" t="n"/>
-      <c r="F15" s="6" t="n"/>
-      <c r="G15" s="6" t="n"/>
-      <c r="H15" s="6" t="n"/>
-      <c r="I15" s="6" t="n"/>
+      <c r="C15" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D15" s="6" t="n">
+        <v>30</v>
+      </c>
+      <c r="E15" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G15" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H15" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I15" s="6" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="16" ht="17" customHeight="1" s="7">
       <c r="B16" s="5" t="inlineStr">
@@ -1376,13 +1544,27 @@
           <t>L03</t>
         </is>
       </c>
-      <c r="C16" s="6" t="n"/>
-      <c r="D16" s="6" t="n"/>
-      <c r="E16" s="6" t="n"/>
-      <c r="F16" s="6" t="n"/>
-      <c r="G16" s="6" t="n"/>
-      <c r="H16" s="6" t="n"/>
-      <c r="I16" s="6" t="n"/>
+      <c r="C16" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D16" s="6" t="n">
+        <v>30</v>
+      </c>
+      <c r="E16" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G16" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H16" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I16" s="6" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="17" ht="17" customHeight="1" s="7">
       <c r="B17" s="5" t="inlineStr">
@@ -1390,13 +1572,27 @@
           <t>L03</t>
         </is>
       </c>
-      <c r="C17" s="6" t="n"/>
-      <c r="D17" s="6" t="n"/>
-      <c r="E17" s="6" t="n"/>
-      <c r="F17" s="6" t="n"/>
-      <c r="G17" s="6" t="n"/>
-      <c r="H17" s="6" t="n"/>
-      <c r="I17" s="6" t="n"/>
+      <c r="C17" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D17" s="6" t="n">
+        <v>30</v>
+      </c>
+      <c r="E17" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G17" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H17" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I17" s="6" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="18" ht="17" customHeight="1" s="7">
       <c r="B18" s="5" t="inlineStr">
@@ -1404,14 +1600,29 @@
           <t>L03</t>
         </is>
       </c>
-      <c r="C18" s="6" t="n"/>
-      <c r="D18" s="6" t="n"/>
-      <c r="E18" s="6" t="n"/>
-      <c r="F18" s="6" t="n"/>
-      <c r="G18" s="6" t="n"/>
-      <c r="H18" s="6" t="n"/>
-      <c r="I18" s="6" t="n"/>
-    </row>
+      <c r="C18" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D18" s="6" t="n">
+        <v>30</v>
+      </c>
+      <c r="E18" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F18" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G18" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H18" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I18" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="B2:D2"/>
@@ -1429,9 +1640,7 @@
   </sheetPr>
   <dimension ref="A1:A1"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14"/>
-  <sheetData>
-    <row r="1"/>
-  </sheetData>
+  <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" paperSize="9"/>
 </worksheet>
@@ -1445,9 +1654,7 @@
   </sheetPr>
   <dimension ref="A1:A1"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14"/>
-  <sheetData>
-    <row r="1"/>
-  </sheetData>
+  <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" paperSize="9"/>
 </worksheet>
@@ -1459,7 +1666,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G45"/>
+  <dimension ref="A1:G44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" style="7" min="1" max="1"/>
@@ -1567,14 +1774,14 @@
       </c>
       <c r="B10" s="14" t="inlineStr">
         <is>
-          <t>99.01%</t>
+          <t>99.0099%</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="13" t="inlineStr">
         <is>
-          <t>Waste Gap Ratio</t>
+          <t>Utilization Gap to 100%</t>
         </is>
       </c>
       <c r="B11" s="14" t="inlineStr">
@@ -1586,252 +1793,262 @@
     <row r="12">
       <c r="A12" s="13" t="inlineStr">
         <is>
-          <t>Utilization Gap to 100%</t>
+          <t>Upper Bound</t>
         </is>
       </c>
       <c r="B12" s="14" t="inlineStr">
         <is>
-          <t>0.9901%</t>
+          <t>1.0000</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="13" t="inlineStr">
         <is>
-          <t>Upper Bound (utilization)</t>
+          <t>Lower Bound</t>
         </is>
       </c>
       <c r="B13" s="14" t="inlineStr">
         <is>
-          <t>1.0 (100%)</t>
+          <t>0.9901</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="13" t="inlineStr">
         <is>
-          <t>Lower Bound</t>
+          <t>Gap</t>
         </is>
       </c>
       <c r="B14" s="14" t="inlineStr">
         <is>
-          <t>0.9901</t>
+          <t>0.9901%</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="13" t="inlineStr">
         <is>
-          <t>Gap</t>
+          <t>Solve Time (s)</t>
         </is>
       </c>
       <c r="B15" s="14" t="inlineStr">
         <is>
-          <t>0.9901%</t>
+          <t>0.16</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="13" t="inlineStr">
         <is>
-          <t>Solve Time (s)</t>
+          <t>Pattern-Library Optimal</t>
         </is>
       </c>
       <c r="B16" s="14" t="inlineStr">
         <is>
-          <t>0.18</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="13" t="inlineStr">
-        <is>
-          <t>Optimality Note</t>
-        </is>
-      </c>
-      <c r="B17" s="14" t="inlineStr">
-        <is>
-          <t>Pattern-library optimal (not necessarily global optimal without complete pattern enumeration)</t>
+          <t>CP-SAT OPTIMAL within generated pattern library</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="12" t="inlineStr">
+        <is>
+          <t>Runtime Breakdown</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="12" t="inlineStr">
-        <is>
-          <t>Runtime Breakdown</t>
+      <c r="A19" s="13" t="inlineStr">
+        <is>
+          <t>pattern_generation_time</t>
+        </is>
+      </c>
+      <c r="B19" s="14" t="inlineStr">
+        <is>
+          <t>94.71s</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="13" t="inlineStr">
         <is>
-          <t>pattern_generation_time</t>
+          <t>master_solve_time</t>
         </is>
       </c>
       <c r="B20" s="14" t="inlineStr">
         <is>
-          <t>1.87s</t>
+          <t>94.78s</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="13" t="inlineStr">
         <is>
-          <t>master_solve_time</t>
+          <t>plotting_time_problem1</t>
         </is>
       </c>
       <c r="B21" s="14" t="inlineStr">
         <is>
-          <t>1.99s</t>
+          <t>9.72s</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="13" t="inlineStr">
         <is>
-          <t>plotting_time_problem1</t>
+          <t>plotting_time_problem2</t>
         </is>
       </c>
       <c r="B22" s="14" t="inlineStr">
         <is>
-          <t>13.38s</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="13" t="inlineStr">
-        <is>
-          <t>plotting_time_problem2</t>
-        </is>
-      </c>
-      <c r="B23" s="14" t="inlineStr">
-        <is>
-          <t>22.28s</t>
+          <t>14.10s</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="12" t="inlineStr">
+        <is>
+          <t>Piece Production Quantities</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="12" t="inlineStr">
-        <is>
-          <t>Piece Production Quantities</t>
+      <c r="A25" s="15" t="inlineStr">
+        <is>
+          <t>Piece</t>
+        </is>
+      </c>
+      <c r="B25" s="15" t="inlineStr">
+        <is>
+          <t>Count</t>
+        </is>
+      </c>
+      <c r="C25" s="15" t="inlineStr">
+        <is>
+          <t>Unit Volume</t>
+        </is>
+      </c>
+      <c r="D25" s="15" t="inlineStr">
+        <is>
+          <t>Total Volume</t>
+        </is>
+      </c>
+      <c r="E25" s="15" t="inlineStr">
+        <is>
+          <t>Unit Profit</t>
+        </is>
+      </c>
+      <c r="F25" s="15" t="inlineStr">
+        <is>
+          <t>Total Profit</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="15" t="inlineStr">
-        <is>
-          <t>Piece</t>
-        </is>
-      </c>
-      <c r="B26" s="15" t="inlineStr">
-        <is>
-          <t>Quantity</t>
-        </is>
-      </c>
-      <c r="C26" s="15" t="inlineStr">
-        <is>
-          <t>Volume/Unit</t>
-        </is>
-      </c>
-      <c r="D26" s="15" t="inlineStr">
-        <is>
-          <t>Total Volume</t>
-        </is>
-      </c>
-      <c r="E26" s="15" t="inlineStr">
-        <is>
-          <t>Unit Profit</t>
-        </is>
-      </c>
-      <c r="F26" s="15" t="inlineStr">
-        <is>
-          <t>Total Profit</t>
-        </is>
+      <c r="A26" s="14" t="inlineStr">
+        <is>
+          <t>J01</t>
+        </is>
+      </c>
+      <c r="B26" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="C26" s="14" t="n">
+        <v>64000</v>
+      </c>
+      <c r="D26" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E26" s="14" t="n">
+        <v>620</v>
+      </c>
+      <c r="F26" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="14" t="inlineStr">
         <is>
-          <t>J01</t>
+          <t>J02</t>
         </is>
       </c>
       <c r="B27" s="14" t="n">
-        <v>0</v>
+        <v>150</v>
       </c>
       <c r="C27" s="14" t="n">
-        <v>64000</v>
+        <v>80000</v>
       </c>
       <c r="D27" s="14" t="n">
-        <v>0</v>
+        <v>12000000</v>
       </c>
       <c r="E27" s="14" t="n">
-        <v>620</v>
+        <v>780</v>
       </c>
       <c r="F27" s="14" t="n">
-        <v>0</v>
+        <v>117000</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="14" t="inlineStr">
         <is>
-          <t>J02</t>
+          <t>J03</t>
         </is>
       </c>
       <c r="B28" s="14" t="n">
-        <v>150</v>
+        <v>700</v>
       </c>
       <c r="C28" s="14" t="n">
-        <v>80000</v>
+        <v>90000</v>
       </c>
       <c r="D28" s="14" t="n">
-        <v>12000000</v>
+        <v>63000000</v>
       </c>
       <c r="E28" s="14" t="n">
-        <v>780</v>
+        <v>880</v>
       </c>
       <c r="F28" s="14" t="n">
-        <v>117000</v>
+        <v>616000</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="14" t="inlineStr">
         <is>
-          <t>J03</t>
+          <t>J04</t>
         </is>
       </c>
       <c r="B29" s="14" t="n">
-        <v>700</v>
+        <v>0</v>
       </c>
       <c r="C29" s="14" t="n">
-        <v>90000</v>
+        <v>180000</v>
       </c>
       <c r="D29" s="14" t="n">
-        <v>63000000</v>
+        <v>0</v>
       </c>
       <c r="E29" s="14" t="n">
-        <v>880</v>
+        <v>1850</v>
       </c>
       <c r="F29" s="14" t="n">
-        <v>616000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="14" t="inlineStr">
         <is>
-          <t>J04</t>
+          <t>J05</t>
         </is>
       </c>
       <c r="B30" s="14" t="n">
         <v>0</v>
       </c>
       <c r="C30" s="14" t="n">
-        <v>180000</v>
+        <v>240000</v>
       </c>
       <c r="D30" s="14" t="n">
         <v>0</v>
       </c>
       <c r="E30" s="14" t="n">
-        <v>1850</v>
+        <v>2520</v>
       </c>
       <c r="F30" s="14" t="n">
         <v>0</v>
@@ -1840,20 +2057,20 @@
     <row r="31">
       <c r="A31" s="14" t="inlineStr">
         <is>
-          <t>J05</t>
+          <t>J06</t>
         </is>
       </c>
       <c r="B31" s="14" t="n">
         <v>0</v>
       </c>
       <c r="C31" s="14" t="n">
-        <v>240000</v>
+        <v>100000</v>
       </c>
       <c r="D31" s="14" t="n">
         <v>0</v>
       </c>
       <c r="E31" s="14" t="n">
-        <v>2520</v>
+        <v>1000</v>
       </c>
       <c r="F31" s="14" t="n">
         <v>0</v>
@@ -1862,278 +2079,256 @@
     <row r="32">
       <c r="A32" s="14" t="inlineStr">
         <is>
-          <t>J06</t>
+          <t>J07</t>
         </is>
       </c>
       <c r="B32" s="14" t="n">
         <v>0</v>
       </c>
       <c r="C32" s="14" t="n">
-        <v>100000</v>
+        <v>48000</v>
       </c>
       <c r="D32" s="14" t="n">
         <v>0</v>
       </c>
       <c r="E32" s="14" t="n">
-        <v>1000</v>
+        <v>540</v>
       </c>
       <c r="F32" s="14" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="14" t="inlineStr">
-        <is>
-          <t>J07</t>
-        </is>
-      </c>
-      <c r="B33" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="C33" s="14" t="n">
-        <v>48000</v>
-      </c>
-      <c r="D33" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="E33" s="14" t="n">
-        <v>540</v>
-      </c>
-      <c r="F33" s="14" t="n">
-        <v>0</v>
+    <row r="34">
+      <c r="A34" s="12" t="inlineStr">
+        <is>
+          <t>Material Utilization Breakdown</t>
+        </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="12" t="inlineStr">
-        <is>
-          <t>Material Utilization Breakdown</t>
+      <c r="A35" s="15" t="inlineStr">
+        <is>
+          <t>Material</t>
+        </is>
+      </c>
+      <c r="B35" s="15" t="inlineStr">
+        <is>
+          <t>Count</t>
+        </is>
+      </c>
+      <c r="C35" s="15" t="inlineStr">
+        <is>
+          <t>Unit Volume</t>
+        </is>
+      </c>
+      <c r="D35" s="15" t="inlineStr">
+        <is>
+          <t>Total Volume</t>
+        </is>
+      </c>
+      <c r="E35" s="15" t="inlineStr">
+        <is>
+          <t>Used Volume</t>
+        </is>
+      </c>
+      <c r="F35" s="15" t="inlineStr">
+        <is>
+          <t>Waste</t>
+        </is>
+      </c>
+      <c r="G35" s="15" t="inlineStr">
+        <is>
+          <t>Utilization</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="15" t="inlineStr">
-        <is>
-          <t>Material</t>
-        </is>
-      </c>
-      <c r="B36" s="15" t="inlineStr">
-        <is>
-          <t>Count</t>
-        </is>
-      </c>
-      <c r="C36" s="15" t="inlineStr">
-        <is>
-          <t>Volume/Material</t>
-        </is>
-      </c>
-      <c r="D36" s="15" t="inlineStr">
-        <is>
-          <t>Total Volume</t>
-        </is>
-      </c>
-      <c r="E36" s="15" t="inlineStr">
-        <is>
-          <t>Used Volume</t>
-        </is>
-      </c>
-      <c r="F36" s="15" t="inlineStr">
-        <is>
-          <t>Waste</t>
-        </is>
-      </c>
-      <c r="G36" s="15" t="inlineStr">
-        <is>
-          <t>Utilization</t>
+      <c r="A36" s="14" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="B36" s="14" t="n">
+        <v>5</v>
+      </c>
+      <c r="C36" s="14" t="n">
+        <v>9000000</v>
+      </c>
+      <c r="D36" s="14" t="n">
+        <v>45000000</v>
+      </c>
+      <c r="E36" s="14" t="n">
+        <v>45000000</v>
+      </c>
+      <c r="F36" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G36" s="14" t="inlineStr">
+        <is>
+          <t>100.00%</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="14" t="inlineStr">
         <is>
-          <t>L01</t>
+          <t>L02</t>
         </is>
       </c>
       <c r="B37" s="14" t="n">
         <v>5</v>
       </c>
       <c r="C37" s="14" t="n">
-        <v>9000000</v>
+        <v>3750000</v>
       </c>
       <c r="D37" s="14" t="n">
-        <v>45000000</v>
+        <v>18750000</v>
       </c>
       <c r="E37" s="14" t="n">
-        <v>45000000</v>
+        <v>18000000</v>
       </c>
       <c r="F37" s="14" t="n">
-        <v>0</v>
+        <v>750000</v>
       </c>
       <c r="G37" s="14" t="inlineStr">
         <is>
-          <t>100.00%</t>
+          <t>96.00%</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="14" t="inlineStr">
         <is>
-          <t>L02</t>
+          <t>L03</t>
         </is>
       </c>
       <c r="B38" s="14" t="n">
         <v>5</v>
       </c>
       <c r="C38" s="14" t="n">
-        <v>3750000</v>
+        <v>2400000</v>
       </c>
       <c r="D38" s="14" t="n">
-        <v>18750000</v>
+        <v>12000000</v>
       </c>
       <c r="E38" s="14" t="n">
-        <v>18000000</v>
+        <v>12000000</v>
       </c>
       <c r="F38" s="14" t="n">
-        <v>750000</v>
+        <v>0</v>
       </c>
       <c r="G38" s="14" t="inlineStr">
         <is>
-          <t>96.00%</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="14" t="inlineStr">
-        <is>
-          <t>L03</t>
-        </is>
-      </c>
-      <c r="B39" s="14" t="n">
+          <t>100.00%</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="12" t="inlineStr">
+        <is>
+          <t>Pattern Usage Details</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="15" t="inlineStr">
+        <is>
+          <t>Pattern ID</t>
+        </is>
+      </c>
+      <c r="B41" s="15" t="inlineStr">
+        <is>
+          <t>Material</t>
+        </is>
+      </c>
+      <c r="C41" s="15" t="inlineStr">
+        <is>
+          <t>Times Used</t>
+        </is>
+      </c>
+      <c r="D41" s="15" t="inlineStr">
+        <is>
+          <t>Pieces</t>
+        </is>
+      </c>
+      <c r="E41" s="15" t="inlineStr">
+        <is>
+          <t>Used Volume</t>
+        </is>
+      </c>
+      <c r="F41" s="15" t="inlineStr">
+        <is>
+          <t>Utilization</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B42" s="14" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="C42" s="14" t="n">
         <v>5</v>
       </c>
-      <c r="C39" s="14" t="n">
-        <v>2400000</v>
-      </c>
-      <c r="D39" s="14" t="n">
-        <v>12000000</v>
-      </c>
-      <c r="E39" s="14" t="n">
-        <v>12000000</v>
-      </c>
-      <c r="F39" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="G39" s="14" t="inlineStr">
+      <c r="D42" s="14" t="n">
+        <v>100</v>
+      </c>
+      <c r="E42" s="14" t="n">
+        <v>9000000</v>
+      </c>
+      <c r="F42" s="14" t="inlineStr">
         <is>
           <t>100.00%</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="12" t="inlineStr">
-        <is>
-          <t>Pattern Usage Details</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="15" t="inlineStr">
-        <is>
-          <t>Pattern ID</t>
-        </is>
-      </c>
-      <c r="B42" s="15" t="inlineStr">
-        <is>
-          <t>Material</t>
-        </is>
-      </c>
-      <c r="C42" s="15" t="inlineStr">
-        <is>
-          <t>Times Used</t>
-        </is>
-      </c>
-      <c r="D42" s="15" t="inlineStr">
-        <is>
-          <t>Pieces</t>
-        </is>
-      </c>
-      <c r="E42" s="15" t="inlineStr">
-        <is>
-          <t>Used Volume</t>
-        </is>
-      </c>
-      <c r="F42" s="15" t="inlineStr">
-        <is>
-          <t>Utilization</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="14" t="n">
-        <v>13</v>
+        <v>97</v>
       </c>
       <c r="B43" s="14" t="inlineStr">
         <is>
-          <t>L01</t>
+          <t>L02</t>
         </is>
       </c>
       <c r="C43" s="14" t="n">
         <v>5</v>
       </c>
       <c r="D43" s="14" t="n">
-        <v>100</v>
+        <v>40</v>
       </c>
       <c r="E43" s="14" t="n">
-        <v>9000000</v>
+        <v>3600000</v>
       </c>
       <c r="F43" s="14" t="inlineStr">
         <is>
-          <t>100.00%</t>
+          <t>96.00%</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="14" t="n">
-        <v>90</v>
+        <v>167</v>
       </c>
       <c r="B44" s="14" t="inlineStr">
         <is>
-          <t>L02</t>
+          <t>L03</t>
         </is>
       </c>
       <c r="C44" s="14" t="n">
         <v>5</v>
       </c>
       <c r="D44" s="14" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="E44" s="14" t="n">
-        <v>3600000</v>
+        <v>2400000</v>
       </c>
       <c r="F44" s="14" t="inlineStr">
-        <is>
-          <t>96.00%</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="14" t="n">
-        <v>153</v>
-      </c>
-      <c r="B45" s="14" t="inlineStr">
-        <is>
-          <t>L03</t>
-        </is>
-      </c>
-      <c r="C45" s="14" t="n">
-        <v>5</v>
-      </c>
-      <c r="D45" s="14" t="n">
-        <v>30</v>
-      </c>
-      <c r="E45" s="14" t="n">
-        <v>2400000</v>
-      </c>
-      <c r="F45" s="14" t="inlineStr">
         <is>
           <t>100.00%</t>
         </is>

</xml_diff>

<commit_message>
Fix: output consistency - ablation CSV, sensitivity P2, seed stability, certificates, runtime naming
- Fix ablation_results.csv: total_used_volume=75000000, num_patterns_used=3 for all
- Extend sensitivity_results.csv: 10 P1 rows + 10 P2 rows
- Extend seed_stability_results.csv: covers both problem1 and problem2
- Fix excel_validation_report.json: now contains both result1 and result2
- Generate all certificate files with honest NOT_PROVED status
- Fix runtime naming: P1/P2 pattern_generation_duration and master_solve_duration
- Regenerate all outputs preserving problem1 (waste=750000) and problem2 (profit=745680)

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/results/result1_filled.xlsx
+++ b/outputs/results/result1_filled.xlsx
@@ -1666,7 +1666,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G44"/>
+  <dimension ref="A1:G46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" style="7" min="1" max="1"/>
@@ -1834,7 +1834,7 @@
       </c>
       <c r="B15" s="14" t="inlineStr">
         <is>
-          <t>0.16</t>
+          <t>0.02</t>
         </is>
       </c>
     </row>
@@ -1860,217 +1860,197 @@
     <row r="19">
       <c r="A19" s="13" t="inlineStr">
         <is>
-          <t>pattern_generation_time</t>
+          <t>problem1_pattern_generation_duration</t>
         </is>
       </c>
       <c r="B19" s="14" t="inlineStr">
         <is>
-          <t>94.71s</t>
+          <t>90.20s</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="13" t="inlineStr">
         <is>
-          <t>master_solve_time</t>
+          <t>problem1_master_solve_duration</t>
         </is>
       </c>
       <c r="B20" s="14" t="inlineStr">
         <is>
-          <t>94.78s</t>
+          <t>90.24s</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="13" t="inlineStr">
         <is>
-          <t>plotting_time_problem1</t>
+          <t>problem1_plotting_duration</t>
         </is>
       </c>
       <c r="B21" s="14" t="inlineStr">
         <is>
-          <t>9.72s</t>
+          <t>8.23s</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="13" t="inlineStr">
         <is>
-          <t>plotting_time_problem2</t>
+          <t>problem2_pattern_generation_duration</t>
         </is>
       </c>
       <c r="B22" s="14" t="inlineStr">
         <is>
-          <t>14.10s</t>
+          <t>87.19s</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="13" t="inlineStr">
+        <is>
+          <t>problem2_master_solve_duration</t>
+        </is>
+      </c>
+      <c r="B23" s="14" t="inlineStr">
+        <is>
+          <t>87.24s</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="12" t="inlineStr">
+      <c r="A24" s="13" t="inlineStr">
+        <is>
+          <t>problem2_plotting_duration</t>
+        </is>
+      </c>
+      <c r="B24" s="14" t="inlineStr">
+        <is>
+          <t>11.87s</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="12" t="inlineStr">
         <is>
           <t>Piece Production Quantities</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="15" t="inlineStr">
+    <row r="27">
+      <c r="A27" s="15" t="inlineStr">
         <is>
           <t>Piece</t>
         </is>
       </c>
-      <c r="B25" s="15" t="inlineStr">
+      <c r="B27" s="15" t="inlineStr">
         <is>
           <t>Count</t>
         </is>
       </c>
-      <c r="C25" s="15" t="inlineStr">
+      <c r="C27" s="15" t="inlineStr">
         <is>
           <t>Unit Volume</t>
         </is>
       </c>
-      <c r="D25" s="15" t="inlineStr">
+      <c r="D27" s="15" t="inlineStr">
         <is>
           <t>Total Volume</t>
         </is>
       </c>
-      <c r="E25" s="15" t="inlineStr">
+      <c r="E27" s="15" t="inlineStr">
         <is>
           <t>Unit Profit</t>
         </is>
       </c>
-      <c r="F25" s="15" t="inlineStr">
+      <c r="F27" s="15" t="inlineStr">
         <is>
           <t>Total Profit</t>
         </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="14" t="inlineStr">
-        <is>
-          <t>J01</t>
-        </is>
-      </c>
-      <c r="B26" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="C26" s="14" t="n">
-        <v>64000</v>
-      </c>
-      <c r="D26" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="E26" s="14" t="n">
-        <v>620</v>
-      </c>
-      <c r="F26" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="14" t="inlineStr">
-        <is>
-          <t>J02</t>
-        </is>
-      </c>
-      <c r="B27" s="14" t="n">
-        <v>150</v>
-      </c>
-      <c r="C27" s="14" t="n">
-        <v>80000</v>
-      </c>
-      <c r="D27" s="14" t="n">
-        <v>12000000</v>
-      </c>
-      <c r="E27" s="14" t="n">
-        <v>780</v>
-      </c>
-      <c r="F27" s="14" t="n">
-        <v>117000</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="14" t="inlineStr">
         <is>
-          <t>J03</t>
+          <t>J01</t>
         </is>
       </c>
       <c r="B28" s="14" t="n">
-        <v>700</v>
+        <v>0</v>
       </c>
       <c r="C28" s="14" t="n">
-        <v>90000</v>
+        <v>64000</v>
       </c>
       <c r="D28" s="14" t="n">
-        <v>63000000</v>
+        <v>0</v>
       </c>
       <c r="E28" s="14" t="n">
-        <v>880</v>
+        <v>620</v>
       </c>
       <c r="F28" s="14" t="n">
-        <v>616000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="14" t="inlineStr">
         <is>
-          <t>J04</t>
+          <t>J02</t>
         </is>
       </c>
       <c r="B29" s="14" t="n">
-        <v>0</v>
+        <v>150</v>
       </c>
       <c r="C29" s="14" t="n">
-        <v>180000</v>
+        <v>80000</v>
       </c>
       <c r="D29" s="14" t="n">
-        <v>0</v>
+        <v>12000000</v>
       </c>
       <c r="E29" s="14" t="n">
-        <v>1850</v>
+        <v>780</v>
       </c>
       <c r="F29" s="14" t="n">
-        <v>0</v>
+        <v>117000</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="14" t="inlineStr">
         <is>
-          <t>J05</t>
+          <t>J03</t>
         </is>
       </c>
       <c r="B30" s="14" t="n">
-        <v>0</v>
+        <v>700</v>
       </c>
       <c r="C30" s="14" t="n">
-        <v>240000</v>
+        <v>90000</v>
       </c>
       <c r="D30" s="14" t="n">
-        <v>0</v>
+        <v>63000000</v>
       </c>
       <c r="E30" s="14" t="n">
-        <v>2520</v>
+        <v>880</v>
       </c>
       <c r="F30" s="14" t="n">
-        <v>0</v>
+        <v>616000</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="14" t="inlineStr">
         <is>
-          <t>J06</t>
+          <t>J04</t>
         </is>
       </c>
       <c r="B31" s="14" t="n">
         <v>0</v>
       </c>
       <c r="C31" s="14" t="n">
-        <v>100000</v>
+        <v>180000</v>
       </c>
       <c r="D31" s="14" t="n">
         <v>0</v>
       </c>
       <c r="E31" s="14" t="n">
-        <v>1000</v>
+        <v>1850</v>
       </c>
       <c r="F31" s="14" t="n">
         <v>0</v>
@@ -2079,256 +2059,300 @@
     <row r="32">
       <c r="A32" s="14" t="inlineStr">
         <is>
+          <t>J05</t>
+        </is>
+      </c>
+      <c r="B32" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="C32" s="14" t="n">
+        <v>240000</v>
+      </c>
+      <c r="D32" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E32" s="14" t="n">
+        <v>2520</v>
+      </c>
+      <c r="F32" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="14" t="inlineStr">
+        <is>
+          <t>J06</t>
+        </is>
+      </c>
+      <c r="B33" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="C33" s="14" t="n">
+        <v>100000</v>
+      </c>
+      <c r="D33" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E33" s="14" t="n">
+        <v>1000</v>
+      </c>
+      <c r="F33" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="14" t="inlineStr">
+        <is>
           <t>J07</t>
         </is>
       </c>
-      <c r="B32" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="C32" s="14" t="n">
+      <c r="B34" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="C34" s="14" t="n">
         <v>48000</v>
       </c>
-      <c r="D32" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="E32" s="14" t="n">
+      <c r="D34" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E34" s="14" t="n">
         <v>540</v>
       </c>
-      <c r="F32" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="12" t="inlineStr">
+      <c r="F34" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="12" t="inlineStr">
         <is>
           <t>Material Utilization Breakdown</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="15" t="inlineStr">
+    <row r="37">
+      <c r="A37" s="15" t="inlineStr">
         <is>
           <t>Material</t>
         </is>
       </c>
-      <c r="B35" s="15" t="inlineStr">
+      <c r="B37" s="15" t="inlineStr">
         <is>
           <t>Count</t>
         </is>
       </c>
-      <c r="C35" s="15" t="inlineStr">
+      <c r="C37" s="15" t="inlineStr">
         <is>
           <t>Unit Volume</t>
         </is>
       </c>
-      <c r="D35" s="15" t="inlineStr">
+      <c r="D37" s="15" t="inlineStr">
         <is>
           <t>Total Volume</t>
         </is>
       </c>
-      <c r="E35" s="15" t="inlineStr">
+      <c r="E37" s="15" t="inlineStr">
         <is>
           <t>Used Volume</t>
         </is>
       </c>
-      <c r="F35" s="15" t="inlineStr">
+      <c r="F37" s="15" t="inlineStr">
         <is>
           <t>Waste</t>
         </is>
       </c>
-      <c r="G35" s="15" t="inlineStr">
+      <c r="G37" s="15" t="inlineStr">
         <is>
           <t>Utilization</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="14" t="inlineStr">
-        <is>
-          <t>L01</t>
-        </is>
-      </c>
-      <c r="B36" s="14" t="n">
-        <v>5</v>
-      </c>
-      <c r="C36" s="14" t="n">
-        <v>9000000</v>
-      </c>
-      <c r="D36" s="14" t="n">
-        <v>45000000</v>
-      </c>
-      <c r="E36" s="14" t="n">
-        <v>45000000</v>
-      </c>
-      <c r="F36" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="G36" s="14" t="inlineStr">
-        <is>
-          <t>100.00%</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="14" t="inlineStr">
-        <is>
-          <t>L02</t>
-        </is>
-      </c>
-      <c r="B37" s="14" t="n">
-        <v>5</v>
-      </c>
-      <c r="C37" s="14" t="n">
-        <v>3750000</v>
-      </c>
-      <c r="D37" s="14" t="n">
-        <v>18750000</v>
-      </c>
-      <c r="E37" s="14" t="n">
-        <v>18000000</v>
-      </c>
-      <c r="F37" s="14" t="n">
-        <v>750000</v>
-      </c>
-      <c r="G37" s="14" t="inlineStr">
-        <is>
-          <t>96.00%</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="14" t="inlineStr">
         <is>
-          <t>L03</t>
+          <t>L01</t>
         </is>
       </c>
       <c r="B38" s="14" t="n">
         <v>5</v>
       </c>
       <c r="C38" s="14" t="n">
+        <v>9000000</v>
+      </c>
+      <c r="D38" s="14" t="n">
+        <v>45000000</v>
+      </c>
+      <c r="E38" s="14" t="n">
+        <v>45000000</v>
+      </c>
+      <c r="F38" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G38" s="14" t="inlineStr">
+        <is>
+          <t>100.00%</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="14" t="inlineStr">
+        <is>
+          <t>L02</t>
+        </is>
+      </c>
+      <c r="B39" s="14" t="n">
+        <v>5</v>
+      </c>
+      <c r="C39" s="14" t="n">
+        <v>3750000</v>
+      </c>
+      <c r="D39" s="14" t="n">
+        <v>18750000</v>
+      </c>
+      <c r="E39" s="14" t="n">
+        <v>18000000</v>
+      </c>
+      <c r="F39" s="14" t="n">
+        <v>750000</v>
+      </c>
+      <c r="G39" s="14" t="inlineStr">
+        <is>
+          <t>96.00%</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="14" t="inlineStr">
+        <is>
+          <t>L03</t>
+        </is>
+      </c>
+      <c r="B40" s="14" t="n">
+        <v>5</v>
+      </c>
+      <c r="C40" s="14" t="n">
         <v>2400000</v>
       </c>
-      <c r="D38" s="14" t="n">
+      <c r="D40" s="14" t="n">
         <v>12000000</v>
       </c>
-      <c r="E38" s="14" t="n">
+      <c r="E40" s="14" t="n">
         <v>12000000</v>
       </c>
-      <c r="F38" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="G38" s="14" t="inlineStr">
+      <c r="F40" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G40" s="14" t="inlineStr">
         <is>
           <t>100.00%</t>
         </is>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" s="12" t="inlineStr">
+    <row r="42">
+      <c r="A42" s="12" t="inlineStr">
         <is>
           <t>Pattern Usage Details</t>
         </is>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" s="15" t="inlineStr">
+    <row r="43">
+      <c r="A43" s="15" t="inlineStr">
         <is>
           <t>Pattern ID</t>
         </is>
       </c>
-      <c r="B41" s="15" t="inlineStr">
+      <c r="B43" s="15" t="inlineStr">
         <is>
           <t>Material</t>
         </is>
       </c>
-      <c r="C41" s="15" t="inlineStr">
+      <c r="C43" s="15" t="inlineStr">
         <is>
           <t>Times Used</t>
         </is>
       </c>
-      <c r="D41" s="15" t="inlineStr">
+      <c r="D43" s="15" t="inlineStr">
         <is>
           <t>Pieces</t>
         </is>
       </c>
-      <c r="E41" s="15" t="inlineStr">
+      <c r="E43" s="15" t="inlineStr">
         <is>
           <t>Used Volume</t>
         </is>
       </c>
-      <c r="F41" s="15" t="inlineStr">
+      <c r="F43" s="15" t="inlineStr">
         <is>
           <t>Utilization</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="14" t="n">
-        <v>13</v>
-      </c>
-      <c r="B42" s="14" t="inlineStr">
-        <is>
-          <t>L01</t>
-        </is>
-      </c>
-      <c r="C42" s="14" t="n">
-        <v>5</v>
-      </c>
-      <c r="D42" s="14" t="n">
-        <v>100</v>
-      </c>
-      <c r="E42" s="14" t="n">
-        <v>9000000</v>
-      </c>
-      <c r="F42" s="14" t="inlineStr">
-        <is>
-          <t>100.00%</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="14" t="n">
-        <v>97</v>
-      </c>
-      <c r="B43" s="14" t="inlineStr">
-        <is>
-          <t>L02</t>
-        </is>
-      </c>
-      <c r="C43" s="14" t="n">
-        <v>5</v>
-      </c>
-      <c r="D43" s="14" t="n">
-        <v>40</v>
-      </c>
-      <c r="E43" s="14" t="n">
-        <v>3600000</v>
-      </c>
-      <c r="F43" s="14" t="inlineStr">
-        <is>
-          <t>96.00%</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="14" t="n">
-        <v>167</v>
+        <v>13</v>
       </c>
       <c r="B44" s="14" t="inlineStr">
         <is>
-          <t>L03</t>
+          <t>L01</t>
         </is>
       </c>
       <c r="C44" s="14" t="n">
         <v>5</v>
       </c>
       <c r="D44" s="14" t="n">
+        <v>100</v>
+      </c>
+      <c r="E44" s="14" t="n">
+        <v>9000000</v>
+      </c>
+      <c r="F44" s="14" t="inlineStr">
+        <is>
+          <t>100.00%</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="14" t="n">
+        <v>97</v>
+      </c>
+      <c r="B45" s="14" t="inlineStr">
+        <is>
+          <t>L02</t>
+        </is>
+      </c>
+      <c r="C45" s="14" t="n">
+        <v>5</v>
+      </c>
+      <c r="D45" s="14" t="n">
+        <v>40</v>
+      </c>
+      <c r="E45" s="14" t="n">
+        <v>3600000</v>
+      </c>
+      <c r="F45" s="14" t="inlineStr">
+        <is>
+          <t>96.00%</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="14" t="n">
+        <v>167</v>
+      </c>
+      <c r="B46" s="14" t="inlineStr">
+        <is>
+          <t>L03</t>
+        </is>
+      </c>
+      <c r="C46" s="14" t="n">
+        <v>5</v>
+      </c>
+      <c r="D46" s="14" t="n">
         <v>30</v>
       </c>
-      <c r="E44" s="14" t="n">
+      <c r="E46" s="14" t="n">
         <v>2400000</v>
       </c>
-      <c r="F44" s="14" t="inlineStr">
+      <c r="F46" s="14" t="inlineStr">
         <is>
           <t>100.00%</t>
         </is>

</xml_diff>

<commit_message>
Improve: Problem 2 748640, Problem 3 order selection idea, docs update
- Problem 2: improved from 745680 to 748640 via balanced weights + expanded exploration (beam_width=10, restarts=20, seed=9999)
- Problem 3: add order selection decision model report, analysis script, and recommendation (H03 recommended)
- Config: problem2.yaml updated with optimized extreme_point parameters
- Docs: README.md, claude.md, experiment_summary.md updated with P3 references and new P2 result
- Excel: both templates validated (metrics_match_json=true, no errors)
- All outputs regenerated: figures, reports, certificates, CSV summaries

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/results/result1_filled.xlsx
+++ b/outputs/results/result1_filled.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" windowWidth="24750" windowHeight="12080" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Sheet2" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Sheet3" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="computed_solution" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet2" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet3" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="computed_solution" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -1666,7 +1666,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G46"/>
+  <dimension ref="A1:G38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" style="7" min="1" max="1"/>
@@ -1853,506 +1853,427 @@
     <row r="18">
       <c r="A18" s="12" t="inlineStr">
         <is>
-          <t>Runtime Breakdown</t>
+          <t>Piece Production Quantities</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="13" t="inlineStr">
-        <is>
-          <t>problem1_pattern_generation_duration</t>
-        </is>
-      </c>
-      <c r="B19" s="14" t="inlineStr">
-        <is>
-          <t>90.20s</t>
+      <c r="A19" s="15" t="inlineStr">
+        <is>
+          <t>Piece</t>
+        </is>
+      </c>
+      <c r="B19" s="15" t="inlineStr">
+        <is>
+          <t>Count</t>
+        </is>
+      </c>
+      <c r="C19" s="15" t="inlineStr">
+        <is>
+          <t>Unit Volume</t>
+        </is>
+      </c>
+      <c r="D19" s="15" t="inlineStr">
+        <is>
+          <t>Total Volume</t>
+        </is>
+      </c>
+      <c r="E19" s="15" t="inlineStr">
+        <is>
+          <t>Unit Profit</t>
+        </is>
+      </c>
+      <c r="F19" s="15" t="inlineStr">
+        <is>
+          <t>Total Profit</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="13" t="inlineStr">
-        <is>
-          <t>problem1_master_solve_duration</t>
-        </is>
-      </c>
-      <c r="B20" s="14" t="inlineStr">
-        <is>
-          <t>90.24s</t>
-        </is>
+      <c r="A20" s="14" t="inlineStr">
+        <is>
+          <t>J01</t>
+        </is>
+      </c>
+      <c r="B20" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="C20" s="14" t="n">
+        <v>64000</v>
+      </c>
+      <c r="D20" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E20" s="14" t="n">
+        <v>620</v>
+      </c>
+      <c r="F20" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="13" t="inlineStr">
-        <is>
-          <t>problem1_plotting_duration</t>
-        </is>
-      </c>
-      <c r="B21" s="14" t="inlineStr">
-        <is>
-          <t>8.23s</t>
-        </is>
+      <c r="A21" s="14" t="inlineStr">
+        <is>
+          <t>J02</t>
+        </is>
+      </c>
+      <c r="B21" s="14" t="n">
+        <v>150</v>
+      </c>
+      <c r="C21" s="14" t="n">
+        <v>80000</v>
+      </c>
+      <c r="D21" s="14" t="n">
+        <v>12000000</v>
+      </c>
+      <c r="E21" s="14" t="n">
+        <v>780</v>
+      </c>
+      <c r="F21" s="14" t="n">
+        <v>117000</v>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="13" t="inlineStr">
-        <is>
-          <t>problem2_pattern_generation_duration</t>
-        </is>
-      </c>
-      <c r="B22" s="14" t="inlineStr">
-        <is>
-          <t>87.19s</t>
-        </is>
+      <c r="A22" s="14" t="inlineStr">
+        <is>
+          <t>J03</t>
+        </is>
+      </c>
+      <c r="B22" s="14" t="n">
+        <v>700</v>
+      </c>
+      <c r="C22" s="14" t="n">
+        <v>90000</v>
+      </c>
+      <c r="D22" s="14" t="n">
+        <v>63000000</v>
+      </c>
+      <c r="E22" s="14" t="n">
+        <v>880</v>
+      </c>
+      <c r="F22" s="14" t="n">
+        <v>616000</v>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="13" t="inlineStr">
-        <is>
-          <t>problem2_master_solve_duration</t>
-        </is>
-      </c>
-      <c r="B23" s="14" t="inlineStr">
-        <is>
-          <t>87.24s</t>
-        </is>
+      <c r="A23" s="14" t="inlineStr">
+        <is>
+          <t>J04</t>
+        </is>
+      </c>
+      <c r="B23" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="C23" s="14" t="n">
+        <v>180000</v>
+      </c>
+      <c r="D23" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E23" s="14" t="n">
+        <v>1850</v>
+      </c>
+      <c r="F23" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="13" t="inlineStr">
-        <is>
-          <t>problem2_plotting_duration</t>
-        </is>
-      </c>
-      <c r="B24" s="14" t="inlineStr">
-        <is>
-          <t>11.87s</t>
-        </is>
+      <c r="A24" s="14" t="inlineStr">
+        <is>
+          <t>J05</t>
+        </is>
+      </c>
+      <c r="B24" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="C24" s="14" t="n">
+        <v>240000</v>
+      </c>
+      <c r="D24" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E24" s="14" t="n">
+        <v>2520</v>
+      </c>
+      <c r="F24" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="14" t="inlineStr">
+        <is>
+          <t>J06</t>
+        </is>
+      </c>
+      <c r="B25" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="C25" s="14" t="n">
+        <v>100000</v>
+      </c>
+      <c r="D25" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E25" s="14" t="n">
+        <v>1000</v>
+      </c>
+      <c r="F25" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="12" t="inlineStr">
-        <is>
-          <t>Piece Production Quantities</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="15" t="inlineStr">
-        <is>
-          <t>Piece</t>
-        </is>
-      </c>
-      <c r="B27" s="15" t="inlineStr">
+      <c r="A26" s="14" t="inlineStr">
+        <is>
+          <t>J07</t>
+        </is>
+      </c>
+      <c r="B26" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="C26" s="14" t="n">
+        <v>48000</v>
+      </c>
+      <c r="D26" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E26" s="14" t="n">
+        <v>540</v>
+      </c>
+      <c r="F26" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="12" t="inlineStr">
+        <is>
+          <t>Material Utilization Breakdown</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="15" t="inlineStr">
+        <is>
+          <t>Material</t>
+        </is>
+      </c>
+      <c r="B29" s="15" t="inlineStr">
         <is>
           <t>Count</t>
         </is>
       </c>
-      <c r="C27" s="15" t="inlineStr">
+      <c r="C29" s="15" t="inlineStr">
         <is>
           <t>Unit Volume</t>
         </is>
       </c>
-      <c r="D27" s="15" t="inlineStr">
+      <c r="D29" s="15" t="inlineStr">
         <is>
           <t>Total Volume</t>
         </is>
       </c>
-      <c r="E27" s="15" t="inlineStr">
-        <is>
-          <t>Unit Profit</t>
-        </is>
-      </c>
-      <c r="F27" s="15" t="inlineStr">
-        <is>
-          <t>Total Profit</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="14" t="inlineStr">
-        <is>
-          <t>J01</t>
-        </is>
-      </c>
-      <c r="B28" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="C28" s="14" t="n">
-        <v>64000</v>
-      </c>
-      <c r="D28" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="E28" s="14" t="n">
-        <v>620</v>
-      </c>
-      <c r="F28" s="14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="14" t="inlineStr">
-        <is>
-          <t>J02</t>
-        </is>
-      </c>
-      <c r="B29" s="14" t="n">
-        <v>150</v>
-      </c>
-      <c r="C29" s="14" t="n">
-        <v>80000</v>
-      </c>
-      <c r="D29" s="14" t="n">
-        <v>12000000</v>
-      </c>
-      <c r="E29" s="14" t="n">
-        <v>780</v>
-      </c>
-      <c r="F29" s="14" t="n">
-        <v>117000</v>
+      <c r="E29" s="15" t="inlineStr">
+        <is>
+          <t>Used Volume</t>
+        </is>
+      </c>
+      <c r="F29" s="15" t="inlineStr">
+        <is>
+          <t>Waste</t>
+        </is>
+      </c>
+      <c r="G29" s="15" t="inlineStr">
+        <is>
+          <t>Utilization</t>
+        </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="14" t="inlineStr">
         <is>
-          <t>J03</t>
+          <t>L01</t>
         </is>
       </c>
       <c r="B30" s="14" t="n">
-        <v>700</v>
+        <v>5</v>
       </c>
       <c r="C30" s="14" t="n">
-        <v>90000</v>
+        <v>9000000</v>
       </c>
       <c r="D30" s="14" t="n">
-        <v>63000000</v>
+        <v>45000000</v>
       </c>
       <c r="E30" s="14" t="n">
-        <v>880</v>
+        <v>45000000</v>
       </c>
       <c r="F30" s="14" t="n">
-        <v>616000</v>
+        <v>0</v>
+      </c>
+      <c r="G30" s="14" t="inlineStr">
+        <is>
+          <t>100.00%</t>
+        </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="14" t="inlineStr">
         <is>
-          <t>J04</t>
+          <t>L02</t>
         </is>
       </c>
       <c r="B31" s="14" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="C31" s="14" t="n">
-        <v>180000</v>
+        <v>3750000</v>
       </c>
       <c r="D31" s="14" t="n">
-        <v>0</v>
+        <v>18750000</v>
       </c>
       <c r="E31" s="14" t="n">
-        <v>1850</v>
+        <v>18000000</v>
       </c>
       <c r="F31" s="14" t="n">
-        <v>0</v>
+        <v>750000</v>
+      </c>
+      <c r="G31" s="14" t="inlineStr">
+        <is>
+          <t>96.00%</t>
+        </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="14" t="inlineStr">
         <is>
-          <t>J05</t>
+          <t>L03</t>
         </is>
       </c>
       <c r="B32" s="14" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="C32" s="14" t="n">
-        <v>240000</v>
+        <v>2400000</v>
       </c>
       <c r="D32" s="14" t="n">
-        <v>0</v>
+        <v>12000000</v>
       </c>
       <c r="E32" s="14" t="n">
-        <v>2520</v>
+        <v>12000000</v>
       </c>
       <c r="F32" s="14" t="n">
         <v>0</v>
       </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="14" t="inlineStr">
-        <is>
-          <t>J06</t>
-        </is>
-      </c>
-      <c r="B33" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="C33" s="14" t="n">
-        <v>100000</v>
-      </c>
-      <c r="D33" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="E33" s="14" t="n">
-        <v>1000</v>
-      </c>
-      <c r="F33" s="14" t="n">
-        <v>0</v>
+      <c r="G32" s="14" t="inlineStr">
+        <is>
+          <t>100.00%</t>
+        </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="14" t="inlineStr">
-        <is>
-          <t>J07</t>
-        </is>
-      </c>
-      <c r="B34" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="C34" s="14" t="n">
-        <v>48000</v>
-      </c>
-      <c r="D34" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="E34" s="14" t="n">
-        <v>540</v>
-      </c>
-      <c r="F34" s="14" t="n">
-        <v>0</v>
+      <c r="A34" s="12" t="inlineStr">
+        <is>
+          <t>Pattern Usage Details</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="15" t="inlineStr">
+        <is>
+          <t>Pattern ID</t>
+        </is>
+      </c>
+      <c r="B35" s="15" t="inlineStr">
+        <is>
+          <t>Material</t>
+        </is>
+      </c>
+      <c r="C35" s="15" t="inlineStr">
+        <is>
+          <t>Times Used</t>
+        </is>
+      </c>
+      <c r="D35" s="15" t="inlineStr">
+        <is>
+          <t>Pieces</t>
+        </is>
+      </c>
+      <c r="E35" s="15" t="inlineStr">
+        <is>
+          <t>Used Volume</t>
+        </is>
+      </c>
+      <c r="F35" s="15" t="inlineStr">
+        <is>
+          <t>Utilization</t>
+        </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="12" t="inlineStr">
-        <is>
-          <t>Material Utilization Breakdown</t>
+      <c r="A36" s="14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B36" s="14" t="inlineStr">
+        <is>
+          <t>L01</t>
+        </is>
+      </c>
+      <c r="C36" s="14" t="n">
+        <v>5</v>
+      </c>
+      <c r="D36" s="14" t="n">
+        <v>100</v>
+      </c>
+      <c r="E36" s="14" t="n">
+        <v>9000000</v>
+      </c>
+      <c r="F36" s="14" t="inlineStr">
+        <is>
+          <t>100.00%</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="15" t="inlineStr">
-        <is>
-          <t>Material</t>
-        </is>
-      </c>
-      <c r="B37" s="15" t="inlineStr">
-        <is>
-          <t>Count</t>
-        </is>
-      </c>
-      <c r="C37" s="15" t="inlineStr">
-        <is>
-          <t>Unit Volume</t>
-        </is>
-      </c>
-      <c r="D37" s="15" t="inlineStr">
-        <is>
-          <t>Total Volume</t>
-        </is>
-      </c>
-      <c r="E37" s="15" t="inlineStr">
-        <is>
-          <t>Used Volume</t>
-        </is>
-      </c>
-      <c r="F37" s="15" t="inlineStr">
-        <is>
-          <t>Waste</t>
-        </is>
-      </c>
-      <c r="G37" s="15" t="inlineStr">
-        <is>
-          <t>Utilization</t>
+      <c r="A37" s="14" t="n">
+        <v>97</v>
+      </c>
+      <c r="B37" s="14" t="inlineStr">
+        <is>
+          <t>L02</t>
+        </is>
+      </c>
+      <c r="C37" s="14" t="n">
+        <v>5</v>
+      </c>
+      <c r="D37" s="14" t="n">
+        <v>40</v>
+      </c>
+      <c r="E37" s="14" t="n">
+        <v>3600000</v>
+      </c>
+      <c r="F37" s="14" t="inlineStr">
+        <is>
+          <t>96.00%</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="14" t="inlineStr">
-        <is>
-          <t>L01</t>
-        </is>
-      </c>
-      <c r="B38" s="14" t="n">
+      <c r="A38" s="14" t="n">
+        <v>167</v>
+      </c>
+      <c r="B38" s="14" t="inlineStr">
+        <is>
+          <t>L03</t>
+        </is>
+      </c>
+      <c r="C38" s="14" t="n">
         <v>5</v>
       </c>
-      <c r="C38" s="14" t="n">
-        <v>9000000</v>
-      </c>
       <c r="D38" s="14" t="n">
-        <v>45000000</v>
+        <v>30</v>
       </c>
       <c r="E38" s="14" t="n">
-        <v>45000000</v>
-      </c>
-      <c r="F38" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="G38" s="14" t="inlineStr">
-        <is>
-          <t>100.00%</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="14" t="inlineStr">
-        <is>
-          <t>L02</t>
-        </is>
-      </c>
-      <c r="B39" s="14" t="n">
-        <v>5</v>
-      </c>
-      <c r="C39" s="14" t="n">
-        <v>3750000</v>
-      </c>
-      <c r="D39" s="14" t="n">
-        <v>18750000</v>
-      </c>
-      <c r="E39" s="14" t="n">
-        <v>18000000</v>
-      </c>
-      <c r="F39" s="14" t="n">
-        <v>750000</v>
-      </c>
-      <c r="G39" s="14" t="inlineStr">
-        <is>
-          <t>96.00%</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="14" t="inlineStr">
-        <is>
-          <t>L03</t>
-        </is>
-      </c>
-      <c r="B40" s="14" t="n">
-        <v>5</v>
-      </c>
-      <c r="C40" s="14" t="n">
         <v>2400000</v>
       </c>
-      <c r="D40" s="14" t="n">
-        <v>12000000</v>
-      </c>
-      <c r="E40" s="14" t="n">
-        <v>12000000</v>
-      </c>
-      <c r="F40" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="G40" s="14" t="inlineStr">
-        <is>
-          <t>100.00%</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="12" t="inlineStr">
-        <is>
-          <t>Pattern Usage Details</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="15" t="inlineStr">
-        <is>
-          <t>Pattern ID</t>
-        </is>
-      </c>
-      <c r="B43" s="15" t="inlineStr">
-        <is>
-          <t>Material</t>
-        </is>
-      </c>
-      <c r="C43" s="15" t="inlineStr">
-        <is>
-          <t>Times Used</t>
-        </is>
-      </c>
-      <c r="D43" s="15" t="inlineStr">
-        <is>
-          <t>Pieces</t>
-        </is>
-      </c>
-      <c r="E43" s="15" t="inlineStr">
-        <is>
-          <t>Used Volume</t>
-        </is>
-      </c>
-      <c r="F43" s="15" t="inlineStr">
-        <is>
-          <t>Utilization</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="14" t="n">
-        <v>13</v>
-      </c>
-      <c r="B44" s="14" t="inlineStr">
-        <is>
-          <t>L01</t>
-        </is>
-      </c>
-      <c r="C44" s="14" t="n">
-        <v>5</v>
-      </c>
-      <c r="D44" s="14" t="n">
-        <v>100</v>
-      </c>
-      <c r="E44" s="14" t="n">
-        <v>9000000</v>
-      </c>
-      <c r="F44" s="14" t="inlineStr">
-        <is>
-          <t>100.00%</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="14" t="n">
-        <v>97</v>
-      </c>
-      <c r="B45" s="14" t="inlineStr">
-        <is>
-          <t>L02</t>
-        </is>
-      </c>
-      <c r="C45" s="14" t="n">
-        <v>5</v>
-      </c>
-      <c r="D45" s="14" t="n">
-        <v>40</v>
-      </c>
-      <c r="E45" s="14" t="n">
-        <v>3600000</v>
-      </c>
-      <c r="F45" s="14" t="inlineStr">
-        <is>
-          <t>96.00%</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="14" t="n">
-        <v>167</v>
-      </c>
-      <c r="B46" s="14" t="inlineStr">
-        <is>
-          <t>L03</t>
-        </is>
-      </c>
-      <c r="C46" s="14" t="n">
-        <v>5</v>
-      </c>
-      <c r="D46" s="14" t="n">
-        <v>30</v>
-      </c>
-      <c r="E46" s="14" t="n">
-        <v>2400000</v>
-      </c>
-      <c r="F46" s="14" t="inlineStr">
+      <c r="F38" s="14" t="inlineStr">
         <is>
           <t>100.00%</t>
         </is>

</xml_diff>